<commit_message>
Fix asset import template and auto code
</commit_message>
<xml_diff>
--- a/public/templates/template_import_aset.xlsx
+++ b/public/templates/template_import_aset.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\puput\aset-baru\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BCABDB-4774-47D0-AAE3-CD6DBEBB2303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BDE8A98-1D68-4914-A477-DA96E70B06E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,20 +21,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
   <si>
     <t>📋  TEMPLATE IMPORT DATA ASET  —  AssetTrack</t>
   </si>
   <si>
-    <t>Isi data mulai baris ke-5. Jangan hapus atau ubah baris header (baris 4). Kolom A–E wajib diisi.</t>
-  </si>
-  <si>
-    <t>Kode Barang *</t>
-  </si>
-  <si>
-    <t>Nama Aset *</t>
-  </si>
-  <si>
     <t>Kategori *</t>
   </si>
   <si>
@@ -53,12 +44,6 @@
     <t>Harga</t>
   </si>
   <si>
-    <t>ELK-001</t>
-  </si>
-  <si>
-    <t>Laptop Dell Latitude</t>
-  </si>
-  <si>
     <t>Elektronik</t>
   </si>
   <si>
@@ -77,9 +62,6 @@
     <t>2024-01-12</t>
   </si>
   <si>
-    <t>ELK-002</t>
-  </si>
-  <si>
     <t>Monitor Samsung 24"</t>
   </si>
   <si>
@@ -95,9 +77,6 @@
     <t>2024-02-03</t>
   </si>
   <si>
-    <t>FRN-001</t>
-  </si>
-  <si>
     <t>Meja Kerja Kayu Jati</t>
   </si>
   <si>
@@ -119,9 +98,6 @@
     <t>2023-07-15</t>
   </si>
   <si>
-    <t>MSN-001</t>
-  </si>
-  <si>
     <t>Mesin Cetak Offset A3</t>
   </si>
   <si>
@@ -143,9 +119,6 @@
     <t>2022-11-20</t>
   </si>
   <si>
-    <t>KND-001</t>
-  </si>
-  <si>
     <t>Toyota Avanza 2021</t>
   </si>
   <si>
@@ -164,9 +137,6 @@
     <t>2021-09-05</t>
   </si>
   <si>
-    <t>INV-001</t>
-  </si>
-  <si>
     <t>Proyektor Epson EB-X51</t>
   </si>
   <si>
@@ -185,9 +155,6 @@
     <t>2023-03-22</t>
   </si>
   <si>
-    <t>GDG-001</t>
-  </si>
-  <si>
     <t>Forklift Manual 2T</t>
   </si>
   <si>
@@ -221,9 +188,6 @@
     <t>A — Kode Barang *</t>
   </si>
   <si>
-    <t>WAJIB. Kode unik untuk setiap aset. Tidak boleh sama dengan kode yang sudah ada di sistem.</t>
-  </si>
-  <si>
     <t>ELK-001, FRN-002, KND-003</t>
   </si>
   <si>
@@ -330,6 +294,21 @@
   </si>
   <si>
     <t>Stok Saat Ini</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Isi data mulai baris ke-5. Jangan hapus atau ubah baris header (baris 4). Kolom B–E wajib diisi.</t>
+  </si>
+  <si>
+    <t>WAJIB. Kode unik untuk setiap aset. Tidak boleh sama dengan kode yang sudah ada di sistem. Tidak perlu isi manual, kode akan langsung di generate di sistem</t>
+  </si>
+  <si>
+    <t>Nama Barang*</t>
+  </si>
+  <si>
+    <t>Celana Katun</t>
   </si>
 </sst>
 </file>
@@ -511,7 +490,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -566,6 +545,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -885,7 +873,7 @@
   <dimension ref="A1:N31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="14" style="19" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
@@ -895,104 +883,106 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="36" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
     </row>
     <row r="2" spans="1:14" ht="22.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-    </row>
-    <row r="3" spans="1:14" ht="8" customHeight="1" thickBot="1" x14ac:dyDescent="0.5"/>
+      <c r="A2" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+    </row>
+    <row r="3" spans="1:14" ht="8" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A3"/>
+    </row>
     <row r="4" spans="1:14" ht="28.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="F4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="M4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="N4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="L4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="19">
+        <v>1</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="E5" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -1000,33 +990,33 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="N5" s="5">
         <v>12500000</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="6" t="s">
-        <v>18</v>
+      <c r="A6" s="19">
+        <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -1034,33 +1024,33 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="N6" s="7">
         <v>3200000</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="3" t="s">
-        <v>24</v>
+      <c r="A7" s="19">
+        <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -1068,33 +1058,33 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="N7" s="5">
         <v>2800000</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="6" t="s">
-        <v>32</v>
+      <c r="A8" s="19">
+        <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1102,33 +1092,33 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="N8" s="7">
         <v>85000000</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="3" t="s">
-        <v>40</v>
+      <c r="A9" s="19">
+        <v>5</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -1136,33 +1126,33 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="N9" s="5">
         <v>210000000</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="6" t="s">
-        <v>47</v>
+      <c r="A10" s="19">
+        <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1170,33 +1160,33 @@
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="6" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="M10" s="6" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="N10" s="7">
         <v>6500000</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="3" t="s">
-        <v>54</v>
+      <c r="A11" s="19">
+        <v>7</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -1204,17 +1194,17 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="N11" s="5">
         <v>45000000</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="10"/>
+      <c r="A12" s="20"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -1230,7 +1220,7 @@
       <c r="N12" s="10"/>
     </row>
     <row r="13" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="11"/>
+      <c r="A13" s="21"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
@@ -1246,7 +1236,7 @@
       <c r="N13" s="11"/>
     </row>
     <row r="14" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="10"/>
+      <c r="A14" s="20"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
       <c r="D14" s="10"/>
@@ -1262,7 +1252,7 @@
       <c r="N14" s="10"/>
     </row>
     <row r="15" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="11"/>
+      <c r="A15" s="21"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
@@ -1278,7 +1268,7 @@
       <c r="N15" s="11"/>
     </row>
     <row r="16" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="10"/>
+      <c r="A16" s="20"/>
       <c r="B16" s="10"/>
       <c r="C16" s="10"/>
       <c r="D16" s="10"/>
@@ -1294,7 +1284,7 @@
       <c r="N16" s="10"/>
     </row>
     <row r="17" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="11"/>
+      <c r="A17" s="21"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
@@ -1310,7 +1300,7 @@
       <c r="N17" s="11"/>
     </row>
     <row r="18" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="10"/>
+      <c r="A18" s="20"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
@@ -1326,7 +1316,7 @@
       <c r="N18" s="10"/>
     </row>
     <row r="19" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="11"/>
+      <c r="A19" s="21"/>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
       <c r="D19" s="11"/>
@@ -1342,7 +1332,7 @@
       <c r="N19" s="11"/>
     </row>
     <row r="20" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="10"/>
+      <c r="A20" s="20"/>
       <c r="B20" s="10"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
@@ -1358,7 +1348,7 @@
       <c r="N20" s="10"/>
     </row>
     <row r="21" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="11"/>
+      <c r="A21" s="21"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11"/>
       <c r="D21" s="11"/>
@@ -1374,7 +1364,7 @@
       <c r="N21" s="11"/>
     </row>
     <row r="22" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="10"/>
+      <c r="A22" s="20"/>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
@@ -1390,7 +1380,7 @@
       <c r="N22" s="10"/>
     </row>
     <row r="23" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="11"/>
+      <c r="A23" s="21"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
       <c r="D23" s="11"/>
@@ -1406,7 +1396,7 @@
       <c r="N23" s="11"/>
     </row>
     <row r="24" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="10"/>
+      <c r="A24" s="20"/>
       <c r="B24" s="10"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
@@ -1422,7 +1412,7 @@
       <c r="N24" s="10"/>
     </row>
     <row r="25" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="11"/>
+      <c r="A25" s="21"/>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
       <c r="D25" s="11"/>
@@ -1438,7 +1428,7 @@
       <c r="N25" s="11"/>
     </row>
     <row r="26" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A26" s="10"/>
+      <c r="A26" s="20"/>
       <c r="B26" s="10"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -1454,7 +1444,7 @@
       <c r="N26" s="10"/>
     </row>
     <row r="27" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="11"/>
+      <c r="A27" s="21"/>
       <c r="B27" s="11"/>
       <c r="C27" s="11"/>
       <c r="D27" s="11"/>
@@ -1470,7 +1460,7 @@
       <c r="N27" s="11"/>
     </row>
     <row r="28" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A28" s="10"/>
+      <c r="A28" s="20"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
@@ -1486,7 +1476,7 @@
       <c r="N28" s="10"/>
     </row>
     <row r="29" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="11"/>
+      <c r="A29" s="21"/>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
@@ -1502,7 +1492,7 @@
       <c r="N29" s="11"/>
     </row>
     <row r="30" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A30" s="10"/>
+      <c r="A30" s="20"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
@@ -1518,7 +1508,7 @@
       <c r="N30" s="10"/>
     </row>
     <row r="31" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" s="11"/>
+      <c r="A31" s="21"/>
       <c r="B31" s="11"/>
       <c r="C31" s="11"/>
       <c r="D31" s="11"/>
@@ -1542,11 +1532,11 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai Tidak Valid" error="Kondisi harus: &quot;baik&quot;, &quot;rusak&quot;, atau &quot;perbaikan&quot;" sqref="E5:E100" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"baik,rusak,perbaikan"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kategori Tidak Valid" error="Pilih kategori yang tersedia dari dropdown." sqref="C5:C100" xr:uid="{00000000-0002-0000-0000-000001000000}">
-      <formula1>"Elektronik,Mesin Produksi,Furniture,Inventaris Kantor,Peralatan Gudang,Kendaraan"</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1:H1048576" xr:uid="{2DAB1C06-5CC2-427A-A330-9CDD4F74A32A}">
       <formula1>"A, B, ED"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Kategori Tidak Valid" error="Pilih kategori yang tersedia dari dropdown." sqref="C1:C1048576" xr:uid="{5937C058-771A-4544-9B6D-6755658F0123}">
+      <formula1>"Stockload,Elektronik,Mesin Produksi,Furniture,Inventaris Kantor,Peralatan Gudang,Kendaraan"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1565,186 +1555,186 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B1" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
+      <c r="B1" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
     </row>
     <row r="2" spans="2:4" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="3" spans="2:4" ht="24" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B3" s="12" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="13" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="13" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="13" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="13" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>74</v>
+        <v>62</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="13" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="15" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="17" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B11" s="15" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="36" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B12" s="17" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>86</v>
+        <v>74</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>87</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="14" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="14" spans="2:4" ht="26" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
+      <c r="B14" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
     </row>
     <row r="15" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
+      <c r="B15" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" s="23"/>
+      <c r="D15" s="23"/>
     </row>
     <row r="16" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
+      <c r="B16" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
     </row>
     <row r="17" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B17" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
+      <c r="B17" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
     </row>
     <row r="18" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
+      <c r="B18" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
     </row>
     <row r="19" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
+      <c r="B19" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="23"/>
+      <c r="D19" s="23"/>
     </row>
     <row r="20" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
+      <c r="B20" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
     </row>
     <row r="21" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
+      <c r="B21" s="25" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
     </row>
     <row r="22" spans="2:4" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
+      <c r="B22" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>